<commit_message>
Añadir pestaña PRECIO-PLATA para seguimiento semanal del costo
Nueva pestaña con tres herramientas integradas:

1. Precio actual de referencia: celdas de entrada para USD/oz y
   tipo de cambio; calcula automáticamente S//gramo plata 999 y 950;
   compara con el precio real pagado al proveedor (S/18/g actual)

2. Impacto en costos por producto: tabla que muestra cuánto sube
   el costo total de cada joya (CL01, CL02, PL01, PL07, PL08,
   Huellita) si el precio por gramo sube S/1 — con gramos usados,
   diferencia absoluta y porcentaje de impacto sobre el precio de venta

3. Registro semanal: historial de 5 semanas pre-cargado (Abr-May 2026)
   + 8 filas vacías para continuar; fórmula automática de S//g 950
   y variación vs semana anterior; guía de 5 fuentes gratuitas donde
   consultar el precio (Google, Kitco, Investing.com, SBS/SUNAT)

Consejo integrado: revisar precio cada lunes antes de aceptar pedidos.

https://claude.ai/code/session_01N2pUUYM6YDwZq1QrkMxHge
</commit_message>
<xml_diff>
--- a/ENJOYA-CONSOLIDADO-2025-2026.xlsx
+++ b/ENJOYA-CONSOLIDADO-2025-2026.xlsx
@@ -9,11 +9,12 @@
   <sheets>
     <sheet name="INICIO" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="COSTOS-PRODUCTOS" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="PUNTO-EQUILIBRIO" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="VENTAS-INGRESOS" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="GUIA-FORMULAS" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="ESTADO-RESULTADOS" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="FLUJO-EFECTIVO" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="PRECIO-PLATA" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="PUNTO-EQUILIBRIO" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="VENTAS-INGRESOS" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="GUIA-FORMULAS" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="ESTADO-RESULTADOS" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="FLUJO-EFECTIVO" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -22,14 +23,21 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="5">
+  <numFmts count="12">
     <numFmt numFmtId="164" formatCode="&quot;S/&quot;#,##0.00"/>
     <numFmt numFmtId="165" formatCode="0.0&quot;%&quot;"/>
     <numFmt numFmtId="166" formatCode="0.0"/>
     <numFmt numFmtId="167" formatCode="&quot;S/&quot;#,##0.000"/>
     <numFmt numFmtId="168" formatCode="DD/MM/YYYY"/>
+    <numFmt numFmtId="169" formatCode="$#,##0.00"/>
+    <numFmt numFmtId="170" formatCode="0.000"/>
+    <numFmt numFmtId="171" formatCode="&quot;S/&quot;#,##0.0000"/>
+    <numFmt numFmtId="172" formatCode="0.0&quot; g&quot;"/>
+    <numFmt numFmtId="173" formatCode="&quot;+S/&quot;#,##0.00"/>
+    <numFmt numFmtId="174" formatCode="yyyy-mm-dd"/>
+    <numFmt numFmtId="175" formatCode="$#,##0.00; [Red]-$#,##0.00"/>
   </numFmts>
-  <fonts count="27">
+  <fonts count="34">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -181,8 +189,46 @@
       <color rgb="00000000"/>
       <sz val="9"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <color rgb="001F4E79"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <i val="1"/>
+      <color rgb="007F6000"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="001F4E79"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <color rgb="007F6000"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <color rgb="00C00000"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <i val="1"/>
+      <color rgb="001F4E79"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <color rgb="007F6000"/>
+      <sz val="10"/>
+    </font>
   </fonts>
-  <fills count="10">
+  <fills count="11">
     <fill>
       <patternFill/>
     </fill>
@@ -229,8 +275,13 @@
         <fgColor rgb="00FFF2CC"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00EBF3FB"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="7">
+  <borders count="8">
     <border>
       <left/>
       <right/>
@@ -310,11 +361,25 @@
         <color rgb="001F4E79"/>
       </bottom>
     </border>
+    <border>
+      <left style="medium">
+        <color rgb="002E75B6"/>
+      </left>
+      <right style="medium">
+        <color rgb="002E75B6"/>
+      </right>
+      <top style="medium">
+        <color rgb="002E75B6"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="002E75B6"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="128">
+  <cellXfs count="196">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -671,6 +736,208 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="26" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="169" fontId="29" fillId="10" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="170" fontId="29" fillId="10" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="171" fontId="19" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="29" fillId="10" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="23" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="172" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="17" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="173" fontId="10" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="10" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="172" fontId="2" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="2" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="2" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="17" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="173" fontId="10" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="10" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="168" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="169" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="170" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="171" fontId="18" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="168" fontId="2" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="169" fontId="2" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="170" fontId="2" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="175" fontId="2" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="175" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="168" fontId="2" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="169" fontId="5" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="170" fontId="2" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="10" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="175" fontId="2" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="171" fontId="20" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="175" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="171" fontId="20" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="175" fontId="0" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -3475,6 +3742,922 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
+    <tabColor rgb="00C0C0C0"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H48"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="8" customWidth="1" min="1" max="1"/>
+    <col width="13" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="15" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="20" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="22" customHeight="1">
+      <c r="A1" s="128" t="inlineStr">
+        <is>
+          <t>SEGUIMIENTO SEMANAL — PRECIO DE LA PLATA  |  ENJOYA</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="22" customHeight="1">
+      <c r="A2" s="129" t="inlineStr">
+        <is>
+          <t>Las celdas en azul claro son para que ingreses datos. Las celdas blancas se calculan solas con fórmulas.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="22" customHeight="1">
+      <c r="A4" s="130" t="inlineStr">
+        <is>
+          <t>📌  PRECIO ACTUAL DE REFERENCIA  (actualizar cada semana)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="15" customHeight="1">
+      <c r="A5" s="131" t="inlineStr">
+        <is>
+          <t>Fuente recomendada: Google → buscar  'precio plata hoy'  o  kitco.com</t>
+        </is>
+      </c>
+      <c r="B5" s="21" t="n"/>
+      <c r="C5" s="21" t="n"/>
+      <c r="D5" s="21" t="n"/>
+      <c r="E5" s="21" t="n"/>
+    </row>
+    <row r="6" ht="32" customHeight="1">
+      <c r="A6" s="86" t="inlineStr">
+        <is>
+          <t>Campo</t>
+        </is>
+      </c>
+      <c r="B6" s="86" t="inlineStr">
+        <is>
+          <t>Valor (INGRESA TÚ)</t>
+        </is>
+      </c>
+      <c r="C6" s="86" t="inlineStr">
+        <is>
+          <t>Calculado automático</t>
+        </is>
+      </c>
+      <c r="D6" s="86" t="inlineStr">
+        <is>
+          <t>Unidad</t>
+        </is>
+      </c>
+      <c r="E6" s="86" t="inlineStr">
+        <is>
+          <t>Nota</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="22" customHeight="1">
+      <c r="A7" s="132" t="inlineStr">
+        <is>
+          <t>Precio plata internacional</t>
+        </is>
+      </c>
+      <c r="B7" s="133" t="n"/>
+      <c r="C7" s="20" t="n"/>
+      <c r="D7" s="134" t="inlineStr">
+        <is>
+          <t>USD / troy oz</t>
+        </is>
+      </c>
+      <c r="E7" s="135" t="inlineStr">
+        <is>
+          <t>Buscar en Google 'silver price today'</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="22" customHeight="1">
+      <c r="A8" s="136" t="inlineStr">
+        <is>
+          <t>Tipo de cambio USD → PEN</t>
+        </is>
+      </c>
+      <c r="B8" s="137" t="n">
+        <v>3.72</v>
+      </c>
+      <c r="C8" s="77" t="n"/>
+      <c r="D8" s="138" t="inlineStr">
+        <is>
+          <t>S/ por USD</t>
+        </is>
+      </c>
+      <c r="E8" s="139" t="inlineStr">
+        <is>
+          <t>Revisa SUNAT o Google 'tipo cambio hoy'</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="22" customHeight="1">
+      <c r="A9" s="140" t="inlineStr">
+        <is>
+          <t>Precio por gramo (plata 999)</t>
+        </is>
+      </c>
+      <c r="B9" s="141">
+        <f>B7/31.1035*B8</f>
+        <v/>
+      </c>
+      <c r="C9" s="10" t="n"/>
+      <c r="D9" s="142" t="inlineStr">
+        <is>
+          <t>S/ / gramo 999</t>
+        </is>
+      </c>
+      <c r="E9" s="143" t="inlineStr">
+        <is>
+          <t>Pura</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="22" customHeight="1">
+      <c r="A10" s="140" t="inlineStr">
+        <is>
+          <t>Precio por gramo (plata 950)</t>
+        </is>
+      </c>
+      <c r="B10" s="141">
+        <f>B7/31.1035*B8*0.95</f>
+        <v/>
+      </c>
+      <c r="C10" s="10" t="n"/>
+      <c r="D10" s="142" t="inlineStr">
+        <is>
+          <t>S/ / gramo 950</t>
+        </is>
+      </c>
+      <c r="E10" s="143" t="inlineStr">
+        <is>
+          <t>La que usa Enjoya</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="22" customHeight="1">
+      <c r="A11" s="144" t="inlineStr">
+        <is>
+          <t>Precio que pago a proveedor</t>
+        </is>
+      </c>
+      <c r="B11" s="145" t="n">
+        <v>18</v>
+      </c>
+      <c r="C11" s="146" t="n"/>
+      <c r="D11" s="147" t="inlineStr">
+        <is>
+          <t>S/ / gramo</t>
+        </is>
+      </c>
+      <c r="E11" s="148" t="inlineStr">
+        <is>
+          <t>⬅ Actualiza si tu proveedor cambia precio</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="22" customHeight="1">
+      <c r="A12" s="149" t="inlineStr">
+        <is>
+          <t>Comparación: Si el spot internacional (plata 950) sube mucho más que lo que paga a su proveedor (S/18/g actualmente), anticipa que el proveedor subirá precios pronto. Referencia: precio plata 950 en planilla = S/18/g (tomado de la Plantilla Control).</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="22" customHeight="1">
+      <c r="A14" s="130" t="inlineStr">
+        <is>
+          <t>💸  IMPACTO EN COSTOS — ¿Cuánto sube mi costo si cambia el precio de la plata?</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="32" customHeight="1">
+      <c r="A15" s="86" t="inlineStr">
+        <is>
+          <t>Producto</t>
+        </is>
+      </c>
+      <c r="B15" s="86" t="inlineStr">
+        <is>
+          <t>Cod.</t>
+        </is>
+      </c>
+      <c r="C15" s="86" t="inlineStr">
+        <is>
+          <t>Gramos
+plata</t>
+        </is>
+      </c>
+      <c r="D15" s="86" t="inlineStr">
+        <is>
+          <t>Costo dije
+actual S/</t>
+        </is>
+      </c>
+      <c r="E15" s="86" t="inlineStr">
+        <is>
+          <t>% del costo
+total</t>
+        </is>
+      </c>
+      <c r="F15" s="86" t="inlineStr">
+        <is>
+          <t>Si sube +S/1/g
+→ nuevo costo</t>
+        </is>
+      </c>
+      <c r="G15" s="86" t="inlineStr">
+        <is>
+          <t>Diferencia
+S/</t>
+        </is>
+      </c>
+      <c r="H15" s="86" t="inlineStr">
+        <is>
+          <t>% impacto
+en precio</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="18" customHeight="1">
+      <c r="A16" s="150" t="inlineStr">
+        <is>
+          <t>Collar dije circular 1.5cm</t>
+        </is>
+      </c>
+      <c r="B16" s="151" t="inlineStr">
+        <is>
+          <t>CL01</t>
+        </is>
+      </c>
+      <c r="C16" s="152" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="D16" s="153" t="n">
+        <v>27</v>
+      </c>
+      <c r="E16" s="154" t="n">
+        <v>35.2</v>
+      </c>
+      <c r="F16" s="155" t="n">
+        <v>78.16</v>
+      </c>
+      <c r="G16" s="156" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="H16" s="157" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="17" ht="18" customHeight="1">
+      <c r="A17" s="158" t="inlineStr">
+        <is>
+          <t>Collar dije circular 2cm</t>
+        </is>
+      </c>
+      <c r="B17" s="159" t="inlineStr">
+        <is>
+          <t>CL02</t>
+        </is>
+      </c>
+      <c r="C17" s="160" t="n">
+        <v>2</v>
+      </c>
+      <c r="D17" s="161" t="n">
+        <v>36</v>
+      </c>
+      <c r="E17" s="162" t="n">
+        <v>42.5</v>
+      </c>
+      <c r="F17" s="163" t="n">
+        <v>86.66</v>
+      </c>
+      <c r="G17" s="164" t="n">
+        <v>2</v>
+      </c>
+      <c r="H17" s="165" t="n">
+        <v>1.2</v>
+      </c>
+    </row>
+    <row r="18" ht="18" customHeight="1">
+      <c r="A18" s="150" t="inlineStr">
+        <is>
+          <t>Pulsera dije colgante 2cm</t>
+        </is>
+      </c>
+      <c r="B18" s="151" t="inlineStr">
+        <is>
+          <t>PL01</t>
+        </is>
+      </c>
+      <c r="C18" s="152" t="n">
+        <v>1</v>
+      </c>
+      <c r="D18" s="153" t="n">
+        <v>18</v>
+      </c>
+      <c r="E18" s="154" t="n">
+        <v>30.7</v>
+      </c>
+      <c r="F18" s="155" t="n">
+        <v>59.66</v>
+      </c>
+      <c r="G18" s="156" t="n">
+        <v>1</v>
+      </c>
+      <c r="H18" s="157" t="n">
+        <v>1.1</v>
+      </c>
+    </row>
+    <row r="19" ht="18" customHeight="1">
+      <c r="A19" s="158" t="inlineStr">
+        <is>
+          <t>Pulsera hilo negro dije</t>
+        </is>
+      </c>
+      <c r="B19" s="159" t="inlineStr">
+        <is>
+          <t>PL07</t>
+        </is>
+      </c>
+      <c r="C19" s="160" t="n">
+        <v>1.8</v>
+      </c>
+      <c r="D19" s="161" t="n">
+        <v>31</v>
+      </c>
+      <c r="E19" s="162" t="n">
+        <v>43.9</v>
+      </c>
+      <c r="F19" s="163" t="n">
+        <v>72.45999999999999</v>
+      </c>
+      <c r="G19" s="164" t="n">
+        <v>1.8</v>
+      </c>
+      <c r="H19" s="165" t="n">
+        <v>1.2</v>
+      </c>
+    </row>
+    <row r="20" ht="18" customHeight="1">
+      <c r="A20" s="150" t="inlineStr">
+        <is>
+          <t>Pulsera con cadena</t>
+        </is>
+      </c>
+      <c r="B20" s="151" t="inlineStr">
+        <is>
+          <t>PL08</t>
+        </is>
+      </c>
+      <c r="C20" s="152" t="n">
+        <v>1.7</v>
+      </c>
+      <c r="D20" s="153" t="n">
+        <v>30</v>
+      </c>
+      <c r="E20" s="154" t="n">
+        <v>40.2</v>
+      </c>
+      <c r="F20" s="155" t="n">
+        <v>76.36</v>
+      </c>
+      <c r="G20" s="156" t="n">
+        <v>1.7</v>
+      </c>
+      <c r="H20" s="157" t="n">
+        <v>1.1</v>
+      </c>
+    </row>
+    <row r="21" ht="18" customHeight="1">
+      <c r="A21" s="158" t="inlineStr">
+        <is>
+          <t>Pulsera Huellita resina</t>
+        </is>
+      </c>
+      <c r="B21" s="159" t="inlineStr">
+        <is>
+          <t>Huell</t>
+        </is>
+      </c>
+      <c r="C21" s="160" t="n">
+        <v>1.7</v>
+      </c>
+      <c r="D21" s="161" t="n">
+        <v>30</v>
+      </c>
+      <c r="E21" s="162" t="n">
+        <v>54.4</v>
+      </c>
+      <c r="F21" s="163" t="n">
+        <v>56.86</v>
+      </c>
+      <c r="G21" s="164" t="n">
+        <v>1.7</v>
+      </c>
+      <c r="H21" s="165" t="n">
+        <v>1.9</v>
+      </c>
+    </row>
+    <row r="22" ht="22" customHeight="1">
+      <c r="A22" s="166" t="inlineStr">
+        <is>
+          <t>Ejemplo: Si el precio que cobras por gramo de plata sube S/1 (de S/18 a S/19/g), el costo del CL02 (2g) sube S/2, de S/84.66 a S/86.66. Tu margen baja de S/84.34 a S/82.34.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="22" customHeight="1">
+      <c r="A24" s="130" t="inlineStr">
+        <is>
+          <t>📅  REGISTRO SEMANAL  (completa cada semana — puedes añadir más filas)</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="32" customHeight="1">
+      <c r="A25" s="86" t="inlineStr">
+        <is>
+          <t>Semana</t>
+        </is>
+      </c>
+      <c r="B25" s="86" t="inlineStr">
+        <is>
+          <t>Fecha</t>
+        </is>
+      </c>
+      <c r="C25" s="86" t="inlineStr">
+        <is>
+          <t>Precio plata
+USD/oz</t>
+        </is>
+      </c>
+      <c r="D25" s="86" t="inlineStr">
+        <is>
+          <t>Tipo cambio
+USD/PEN</t>
+        </is>
+      </c>
+      <c r="E25" s="86" t="inlineStr">
+        <is>
+          <t>S/ por gramo
+plata 950</t>
+        </is>
+      </c>
+      <c r="F25" s="86" t="inlineStr">
+        <is>
+          <t>Precio proveedor
+S//gramo</t>
+        </is>
+      </c>
+      <c r="G25" s="86" t="inlineStr">
+        <is>
+          <t>Variación
+vs semana ant.</t>
+        </is>
+      </c>
+      <c r="H25" s="86" t="inlineStr">
+        <is>
+          <t>Observación</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="18" customHeight="1">
+      <c r="A26" s="167" t="inlineStr">
+        <is>
+          <t>S1</t>
+        </is>
+      </c>
+      <c r="B26" s="168" t="n">
+        <v>46119</v>
+      </c>
+      <c r="C26" s="169" t="n">
+        <v>32.1</v>
+      </c>
+      <c r="D26" s="170" t="n">
+        <v>3.7</v>
+      </c>
+      <c r="E26" s="171">
+        <f>C26/31.1035*D26*0.95</f>
+        <v/>
+      </c>
+      <c r="F26" s="172" t="n">
+        <v>18</v>
+      </c>
+      <c r="G26" s="20" t="n"/>
+      <c r="H26" s="135" t="inlineStr">
+        <is>
+          <t>Registro inicial</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="18" customHeight="1">
+      <c r="A27" s="173" t="inlineStr">
+        <is>
+          <t>S2</t>
+        </is>
+      </c>
+      <c r="B27" s="174" t="n">
+        <v>46126</v>
+      </c>
+      <c r="C27" s="175" t="n">
+        <v>31.8</v>
+      </c>
+      <c r="D27" s="176" t="n">
+        <v>3.71</v>
+      </c>
+      <c r="E27" s="171">
+        <f>C27/31.1035*D27*0.95</f>
+        <v/>
+      </c>
+      <c r="F27" s="177" t="n">
+        <v>18</v>
+      </c>
+      <c r="G27" s="178">
+        <f>C27-C26</f>
+        <v/>
+      </c>
+      <c r="H27" s="139" t="inlineStr"/>
+    </row>
+    <row r="28" ht="18" customHeight="1">
+      <c r="A28" s="167" t="inlineStr">
+        <is>
+          <t>S3</t>
+        </is>
+      </c>
+      <c r="B28" s="168" t="n">
+        <v>46133</v>
+      </c>
+      <c r="C28" s="169" t="n">
+        <v>32.5</v>
+      </c>
+      <c r="D28" s="170" t="n">
+        <v>3.72</v>
+      </c>
+      <c r="E28" s="171">
+        <f>C28/31.1035*D28*0.95</f>
+        <v/>
+      </c>
+      <c r="F28" s="172" t="n">
+        <v>18</v>
+      </c>
+      <c r="G28" s="179">
+        <f>C28-C27</f>
+        <v/>
+      </c>
+      <c r="H28" s="135" t="inlineStr">
+        <is>
+          <t>Plata sube levemente</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="18" customHeight="1">
+      <c r="A29" s="173" t="inlineStr">
+        <is>
+          <t>S4</t>
+        </is>
+      </c>
+      <c r="B29" s="174" t="n">
+        <v>46140</v>
+      </c>
+      <c r="C29" s="175" t="n">
+        <v>31.5</v>
+      </c>
+      <c r="D29" s="176" t="n">
+        <v>3.72</v>
+      </c>
+      <c r="E29" s="171">
+        <f>C29/31.1035*D29*0.95</f>
+        <v/>
+      </c>
+      <c r="F29" s="177" t="n">
+        <v>18</v>
+      </c>
+      <c r="G29" s="178">
+        <f>C29-C28</f>
+        <v/>
+      </c>
+      <c r="H29" s="139" t="inlineStr"/>
+    </row>
+    <row r="30" ht="18" customHeight="1">
+      <c r="A30" s="180" t="inlineStr">
+        <is>
+          <t>S5</t>
+        </is>
+      </c>
+      <c r="B30" s="181" t="n">
+        <v>46147</v>
+      </c>
+      <c r="C30" s="182" t="n">
+        <v>31.8</v>
+      </c>
+      <c r="D30" s="183" t="n">
+        <v>3.72</v>
+      </c>
+      <c r="E30" s="171">
+        <f>C30/31.1035*D30*0.95</f>
+        <v/>
+      </c>
+      <c r="F30" s="184" t="n">
+        <v>18</v>
+      </c>
+      <c r="G30" s="185">
+        <f>C30-C29</f>
+        <v/>
+      </c>
+      <c r="H30" s="186" t="inlineStr">
+        <is>
+          <t>Semana actual</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="18" customHeight="1">
+      <c r="A31" s="20" t="n"/>
+      <c r="B31" s="20" t="n"/>
+      <c r="C31" s="20" t="n"/>
+      <c r="D31" s="20" t="n"/>
+      <c r="E31" s="187">
+        <f>IF(C31&lt;&gt;"",C31/31.1035*D31*0.95,"")</f>
+        <v/>
+      </c>
+      <c r="F31" s="20" t="n"/>
+      <c r="G31" s="188">
+        <f>IF(C31&lt;&gt;"",C31-C30,"")</f>
+        <v/>
+      </c>
+      <c r="H31" s="20" t="n"/>
+    </row>
+    <row r="32" ht="18" customHeight="1">
+      <c r="A32" s="77" t="n"/>
+      <c r="B32" s="77" t="n"/>
+      <c r="C32" s="77" t="n"/>
+      <c r="D32" s="77" t="n"/>
+      <c r="E32" s="189">
+        <f>IF(C32&lt;&gt;"",C32/31.1035*D32*0.95,"")</f>
+        <v/>
+      </c>
+      <c r="F32" s="77" t="n"/>
+      <c r="G32" s="190">
+        <f>IF(C32&lt;&gt;"",C32-C31,"")</f>
+        <v/>
+      </c>
+      <c r="H32" s="77" t="n"/>
+    </row>
+    <row r="33" ht="18" customHeight="1">
+      <c r="A33" s="20" t="n"/>
+      <c r="B33" s="20" t="n"/>
+      <c r="C33" s="20" t="n"/>
+      <c r="D33" s="20" t="n"/>
+      <c r="E33" s="187">
+        <f>IF(C33&lt;&gt;"",C33/31.1035*D33*0.95,"")</f>
+        <v/>
+      </c>
+      <c r="F33" s="20" t="n"/>
+      <c r="G33" s="188">
+        <f>IF(C33&lt;&gt;"",C33-C32,"")</f>
+        <v/>
+      </c>
+      <c r="H33" s="20" t="n"/>
+    </row>
+    <row r="34" ht="18" customHeight="1">
+      <c r="A34" s="77" t="n"/>
+      <c r="B34" s="77" t="n"/>
+      <c r="C34" s="77" t="n"/>
+      <c r="D34" s="77" t="n"/>
+      <c r="E34" s="189">
+        <f>IF(C34&lt;&gt;"",C34/31.1035*D34*0.95,"")</f>
+        <v/>
+      </c>
+      <c r="F34" s="77" t="n"/>
+      <c r="G34" s="190">
+        <f>IF(C34&lt;&gt;"",C34-C33,"")</f>
+        <v/>
+      </c>
+      <c r="H34" s="77" t="n"/>
+    </row>
+    <row r="35" ht="18" customHeight="1">
+      <c r="A35" s="20" t="n"/>
+      <c r="B35" s="20" t="n"/>
+      <c r="C35" s="20" t="n"/>
+      <c r="D35" s="20" t="n"/>
+      <c r="E35" s="187">
+        <f>IF(C35&lt;&gt;"",C35/31.1035*D35*0.95,"")</f>
+        <v/>
+      </c>
+      <c r="F35" s="20" t="n"/>
+      <c r="G35" s="188">
+        <f>IF(C35&lt;&gt;"",C35-C34,"")</f>
+        <v/>
+      </c>
+      <c r="H35" s="20" t="n"/>
+    </row>
+    <row r="36" ht="18" customHeight="1">
+      <c r="A36" s="77" t="n"/>
+      <c r="B36" s="77" t="n"/>
+      <c r="C36" s="77" t="n"/>
+      <c r="D36" s="77" t="n"/>
+      <c r="E36" s="189">
+        <f>IF(C36&lt;&gt;"",C36/31.1035*D36*0.95,"")</f>
+        <v/>
+      </c>
+      <c r="F36" s="77" t="n"/>
+      <c r="G36" s="190">
+        <f>IF(C36&lt;&gt;"",C36-C35,"")</f>
+        <v/>
+      </c>
+      <c r="H36" s="77" t="n"/>
+    </row>
+    <row r="37" ht="18" customHeight="1">
+      <c r="A37" s="20" t="n"/>
+      <c r="B37" s="20" t="n"/>
+      <c r="C37" s="20" t="n"/>
+      <c r="D37" s="20" t="n"/>
+      <c r="E37" s="187">
+        <f>IF(C37&lt;&gt;"",C37/31.1035*D37*0.95,"")</f>
+        <v/>
+      </c>
+      <c r="F37" s="20" t="n"/>
+      <c r="G37" s="188">
+        <f>IF(C37&lt;&gt;"",C37-C36,"")</f>
+        <v/>
+      </c>
+      <c r="H37" s="20" t="n"/>
+    </row>
+    <row r="38" ht="18" customHeight="1">
+      <c r="A38" s="77" t="n"/>
+      <c r="B38" s="77" t="n"/>
+      <c r="C38" s="77" t="n"/>
+      <c r="D38" s="77" t="n"/>
+      <c r="E38" s="189">
+        <f>IF(C38&lt;&gt;"",C38/31.1035*D38*0.95,"")</f>
+        <v/>
+      </c>
+      <c r="F38" s="77" t="n"/>
+      <c r="G38" s="190">
+        <f>IF(C38&lt;&gt;"",C38-C37,"")</f>
+        <v/>
+      </c>
+      <c r="H38" s="77" t="n"/>
+    </row>
+    <row r="40" ht="22" customHeight="1">
+      <c r="A40" s="130" t="inlineStr">
+        <is>
+          <t>🔍  DÓNDE CONSULTAR EL PRECIO DE LA PLATA (gratis)</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="16" customHeight="1"/>
+    <row r="42" ht="20" customHeight="1">
+      <c r="A42" s="191" t="inlineStr">
+        <is>
+          <t>Google</t>
+        </is>
+      </c>
+      <c r="B42" s="192" t="inlineStr">
+        <is>
+          <t>Buscar: 'precio plata hoy' o 'silver price today'</t>
+        </is>
+      </c>
+      <c r="C42" s="20" t="n"/>
+      <c r="D42" s="20" t="n"/>
+      <c r="E42" s="135" t="inlineStr">
+        <is>
+          <t>Aparece el gráfico directamente en el buscador. Es el más rápido.</t>
+        </is>
+      </c>
+      <c r="F42" s="20" t="n"/>
+      <c r="G42" s="20" t="n"/>
+      <c r="H42" s="20" t="n"/>
+    </row>
+    <row r="43" ht="20" customHeight="1">
+      <c r="A43" s="193" t="inlineStr">
+        <is>
+          <t>Kitco.com</t>
+        </is>
+      </c>
+      <c r="B43" s="194" t="inlineStr">
+        <is>
+          <t>kitco.com → Markets → Silver</t>
+        </is>
+      </c>
+      <c r="C43" s="77" t="n"/>
+      <c r="D43" s="77" t="n"/>
+      <c r="E43" s="139" t="inlineStr">
+        <is>
+          <t>Precio en tiempo real USD/oz. Histórico gratuito.</t>
+        </is>
+      </c>
+      <c r="F43" s="77" t="n"/>
+      <c r="G43" s="77" t="n"/>
+      <c r="H43" s="77" t="n"/>
+    </row>
+    <row r="44" ht="20" customHeight="1">
+      <c r="A44" s="191" t="inlineStr">
+        <is>
+          <t>Investing.com</t>
+        </is>
+      </c>
+      <c r="B44" s="192" t="inlineStr">
+        <is>
+          <t>investing.com → Commodities → Silver</t>
+        </is>
+      </c>
+      <c r="C44" s="20" t="n"/>
+      <c r="D44" s="20" t="n"/>
+      <c r="E44" s="135" t="inlineStr">
+        <is>
+          <t>Precio en USD y gráfico. Puedes ver 1 semana, 1 mes, 1 año.</t>
+        </is>
+      </c>
+      <c r="F44" s="20" t="n"/>
+      <c r="G44" s="20" t="n"/>
+      <c r="H44" s="20" t="n"/>
+    </row>
+    <row r="45" ht="20" customHeight="1">
+      <c r="A45" s="193" t="inlineStr">
+        <is>
+          <t>Google Finance</t>
+        </is>
+      </c>
+      <c r="B45" s="194" t="inlineStr">
+        <is>
+          <t>Buscar: 'XAG USD' en Google</t>
+        </is>
+      </c>
+      <c r="C45" s="77" t="n"/>
+      <c r="D45" s="77" t="n"/>
+      <c r="E45" s="139" t="inlineStr">
+        <is>
+          <t>XAG = símbolo internacional de la plata. Muestra precio al instante.</t>
+        </is>
+      </c>
+      <c r="F45" s="77" t="n"/>
+      <c r="G45" s="77" t="n"/>
+      <c r="H45" s="77" t="n"/>
+    </row>
+    <row r="46" ht="20" customHeight="1">
+      <c r="A46" s="191" t="inlineStr">
+        <is>
+          <t>SBS / SUNAT</t>
+        </is>
+      </c>
+      <c r="B46" s="192" t="inlineStr">
+        <is>
+          <t>sbs.gob.pe o sunat.gob.pe</t>
+        </is>
+      </c>
+      <c r="C46" s="20" t="n"/>
+      <c r="D46" s="20" t="n"/>
+      <c r="E46" s="135" t="inlineStr">
+        <is>
+          <t>Para el tipo de cambio oficial USD → PEN del día.</t>
+        </is>
+      </c>
+      <c r="F46" s="20" t="n"/>
+      <c r="G46" s="20" t="n"/>
+      <c r="H46" s="20" t="n"/>
+    </row>
+    <row r="48" ht="22" customHeight="1">
+      <c r="A48" s="195" t="inlineStr">
+        <is>
+          <t>💡  Consejo práctico: Revisa el precio de la plata cada lunes antes de aceptar pedidos de la semana. Si el spot en USD sube más de 5% en el mes, habla con tu proveedor para confirmar si mantendrá el precio. El precio que paga por el dije (S/18/g actualmente) es tu costo real — el internacional es tu señal de alerta.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="20">
+    <mergeCell ref="B42:D42"/>
+    <mergeCell ref="A48:H48"/>
+    <mergeCell ref="E45:H45"/>
+    <mergeCell ref="A24:H24"/>
+    <mergeCell ref="B44:D44"/>
+    <mergeCell ref="A1:H1"/>
+    <mergeCell ref="E43:H43"/>
+    <mergeCell ref="E42:H42"/>
+    <mergeCell ref="A12:E12"/>
+    <mergeCell ref="B45:D45"/>
+    <mergeCell ref="A2:H2"/>
+    <mergeCell ref="E44:H44"/>
+    <mergeCell ref="A5:E5"/>
+    <mergeCell ref="A14:H14"/>
+    <mergeCell ref="A22:H22"/>
+    <mergeCell ref="A4:E4"/>
+    <mergeCell ref="B46:D46"/>
+    <mergeCell ref="E46:H46"/>
+    <mergeCell ref="B43:D43"/>
+    <mergeCell ref="A40:H40"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
     <tabColor rgb="00FF0000"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
@@ -3982,7 +5165,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="0070AD47"/>
@@ -9691,7 +10874,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="00FFC000"/>
@@ -10259,7 +11442,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="00375623"/>
@@ -11255,6 +12438,15 @@
           <t>ANÁLISIS E INTERPRETACIÓN</t>
         </is>
       </c>
+      <c r="B35" s="79" t="n"/>
+      <c r="C35" s="79" t="n"/>
+      <c r="D35" s="79" t="n"/>
+      <c r="E35" s="79" t="n"/>
+      <c r="F35" s="79" t="n"/>
+      <c r="G35" s="79" t="n"/>
+      <c r="H35" s="79" t="n"/>
+      <c r="I35" s="79" t="n"/>
+      <c r="J35" s="80" t="n"/>
     </row>
     <row r="36" ht="45" customHeight="1">
       <c r="A36" s="120" t="inlineStr">
@@ -11267,6 +12459,14 @@
           <t>Cada sol vendido, S/ 0.48 quedan para cubrir gastos. Esto es saludable para joyería artesanal.</t>
         </is>
       </c>
+      <c r="C36" s="79" t="n"/>
+      <c r="D36" s="79" t="n"/>
+      <c r="E36" s="79" t="n"/>
+      <c r="F36" s="79" t="n"/>
+      <c r="G36" s="79" t="n"/>
+      <c r="H36" s="79" t="n"/>
+      <c r="I36" s="79" t="n"/>
+      <c r="J36" s="80" t="n"/>
     </row>
     <row r="37" ht="45" customHeight="1">
       <c r="A37" s="122" t="inlineStr">
@@ -11279,6 +12479,14 @@
           <t>Los gastos fijos (S/2,797/mes × 16 meses = S/44,752) superan el margen bruto total (S/21,198). Esto refleja que el volumen de ventas aún no alcanza el punto de equilibrio mensual (~33 collares CL02).</t>
         </is>
       </c>
+      <c r="C37" s="79" t="n"/>
+      <c r="D37" s="79" t="n"/>
+      <c r="E37" s="79" t="n"/>
+      <c r="F37" s="79" t="n"/>
+      <c r="G37" s="79" t="n"/>
+      <c r="H37" s="79" t="n"/>
+      <c r="I37" s="79" t="n"/>
+      <c r="J37" s="80" t="n"/>
     </row>
     <row r="38" ht="45" customHeight="1">
       <c r="A38" s="124" t="inlineStr">
@@ -11291,6 +12499,14 @@
           <t>Si la emprendedora no se paga sueldo aún (común en fases iniciales), los gastos operativos reales bajan a S/1,997/mes. Con ese escenario, la utilidad operativa mejora significativamente.</t>
         </is>
       </c>
+      <c r="C38" s="79" t="n"/>
+      <c r="D38" s="79" t="n"/>
+      <c r="E38" s="79" t="n"/>
+      <c r="F38" s="79" t="n"/>
+      <c r="G38" s="79" t="n"/>
+      <c r="H38" s="79" t="n"/>
+      <c r="I38" s="79" t="n"/>
+      <c r="J38" s="80" t="n"/>
     </row>
     <row r="39" ht="45" customHeight="1">
       <c r="A39" s="120" t="inlineStr">
@@ -11303,6 +12519,14 @@
           <t>Mar 2025 (S/5,034), May 2025 (S/4,543) y Dic 2025 (S/6,757) son los meses con mayores ingresos. Dic 2025 probablemente cubrió costos fijos y generó utilidad. Identificar y replicar esos patrones es clave.</t>
         </is>
       </c>
+      <c r="C39" s="79" t="n"/>
+      <c r="D39" s="79" t="n"/>
+      <c r="E39" s="79" t="n"/>
+      <c r="F39" s="79" t="n"/>
+      <c r="G39" s="79" t="n"/>
+      <c r="H39" s="79" t="n"/>
+      <c r="I39" s="79" t="n"/>
+      <c r="J39" s="80" t="n"/>
     </row>
     <row r="40" ht="45" customHeight="1">
       <c r="A40" s="126" t="inlineStr">
@@ -11315,6 +12539,14 @@
           <t>Incrementar volumen: llegar a 35+ pedidos/mes de collares CL01/CL02 garantiza punto de equilibrio. Ferias, temporadas altas y combos son palancas para escalar sin aumentar costos fijos.</t>
         </is>
       </c>
+      <c r="C40" s="79" t="n"/>
+      <c r="D40" s="79" t="n"/>
+      <c r="E40" s="79" t="n"/>
+      <c r="F40" s="79" t="n"/>
+      <c r="G40" s="79" t="n"/>
+      <c r="H40" s="79" t="n"/>
+      <c r="I40" s="79" t="n"/>
+      <c r="J40" s="80" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="14">
@@ -11323,8 +12555,8 @@
     <mergeCell ref="B37:J37"/>
     <mergeCell ref="A17:J17"/>
     <mergeCell ref="A9:J9"/>
+    <mergeCell ref="B36:J36"/>
     <mergeCell ref="A2:J2"/>
-    <mergeCell ref="B36:J36"/>
     <mergeCell ref="A21:J21"/>
     <mergeCell ref="A30:J30"/>
     <mergeCell ref="B40:J40"/>
@@ -11337,7 +12569,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="00F4B942"/>
@@ -12301,6 +13533,15 @@
           <t>INTERPRETACIÓN DEL FLUJO DE EFECTIVO</t>
         </is>
       </c>
+      <c r="B40" s="79" t="n"/>
+      <c r="C40" s="79" t="n"/>
+      <c r="D40" s="79" t="n"/>
+      <c r="E40" s="79" t="n"/>
+      <c r="F40" s="79" t="n"/>
+      <c r="G40" s="79" t="n"/>
+      <c r="H40" s="79" t="n"/>
+      <c r="I40" s="79" t="n"/>
+      <c r="J40" s="80" t="n"/>
     </row>
     <row r="41" ht="45" customHeight="1">
       <c r="A41" s="124" t="inlineStr">
@@ -12313,6 +13554,14 @@
           <t>El flujo operativo negativo acumulado refleja que los costos fijos no se cubren todos los meses. Sin embargo, en meses de alta venta (Mar/May 2025, Dic 2025) el flujo puede ser positivo.</t>
         </is>
       </c>
+      <c r="C41" s="79" t="n"/>
+      <c r="D41" s="79" t="n"/>
+      <c r="E41" s="79" t="n"/>
+      <c r="F41" s="79" t="n"/>
+      <c r="G41" s="79" t="n"/>
+      <c r="H41" s="79" t="n"/>
+      <c r="I41" s="79" t="n"/>
+      <c r="J41" s="80" t="n"/>
     </row>
     <row r="42" ht="45" customHeight="1">
       <c r="A42" s="122" t="inlineStr">
@@ -12325,6 +13574,14 @@
           <t>Ingresos muy bajos vs costos fijos de S/2,797. Estos meses requieren reserva de efectivo o reducción temporal de gastos.</t>
         </is>
       </c>
+      <c r="C42" s="79" t="n"/>
+      <c r="D42" s="79" t="n"/>
+      <c r="E42" s="79" t="n"/>
+      <c r="F42" s="79" t="n"/>
+      <c r="G42" s="79" t="n"/>
+      <c r="H42" s="79" t="n"/>
+      <c r="I42" s="79" t="n"/>
+      <c r="J42" s="80" t="n"/>
     </row>
     <row r="43" ht="45" customHeight="1">
       <c r="A43" s="120" t="inlineStr">
@@ -12337,6 +13594,14 @@
           <t>Con S/6,757 de ingresos y S/2,797 de costos fijos, el flujo neto de Dic 2025 es positivo. Estrategia: preparar inventario en noviembre para capitalizar la temporada navideña.</t>
         </is>
       </c>
+      <c r="C43" s="79" t="n"/>
+      <c r="D43" s="79" t="n"/>
+      <c r="E43" s="79" t="n"/>
+      <c r="F43" s="79" t="n"/>
+      <c r="G43" s="79" t="n"/>
+      <c r="H43" s="79" t="n"/>
+      <c r="I43" s="79" t="n"/>
+      <c r="J43" s="80" t="n"/>
     </row>
     <row r="44" ht="45" customHeight="1">
       <c r="A44" s="126" t="inlineStr">
@@ -12349,6 +13614,14 @@
           <t>Los clientes pagan separaciones (depósitos) antes de recibir la joya. Esto mejora el flujo de caja real. Oct-Abr se registraron S/5,060 en separaciones cobradas por adelantado.</t>
         </is>
       </c>
+      <c r="C44" s="79" t="n"/>
+      <c r="D44" s="79" t="n"/>
+      <c r="E44" s="79" t="n"/>
+      <c r="F44" s="79" t="n"/>
+      <c r="G44" s="79" t="n"/>
+      <c r="H44" s="79" t="n"/>
+      <c r="I44" s="79" t="n"/>
+      <c r="J44" s="80" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="14">

</xml_diff>